<commit_message>
Design re-structure, now using device sheets. Power and BMS boards completed.
</commit_message>
<xml_diff>
--- a/electronics/pcb_files/board_files/Pack_BMS_Module/Project Outputs/Project Exports/Bill of Materials.xlsx
+++ b/electronics/pcb_files/board_files/Pack_BMS_Module/Project Outputs/Project Exports/Bill of Materials.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="133">
   <si>
     <t>Project File Name:</t>
   </si>
@@ -50,367 +50,382 @@
     <t xml:space="preserve">Date Exported: </t>
   </si>
   <si>
+    <t>1µF</t>
+  </si>
+  <si>
+    <t>25V</t>
+  </si>
+  <si>
+    <t>Amber</t>
+  </si>
+  <si>
+    <t>CONN PLUG 10POS 2.50MM R/A SLDR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Variant: </t>
+  </si>
+  <si>
+    <t>Part Number</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Tolerance</t>
+  </si>
+  <si>
+    <t>Voltage</t>
+  </si>
+  <si>
+    <t>Color</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Manufacturer</t>
+  </si>
+  <si>
+    <t>Supplier</t>
+  </si>
+  <si>
+    <t>Supplier Part Number</t>
+  </si>
+  <si>
+    <t>±10%</t>
+  </si>
+  <si>
+    <t>TE Connectivity AMP Connectors</t>
+  </si>
+  <si>
+    <t>The ROS Robot Project</t>
+  </si>
+  <si>
+    <t>Pack_BMS_Module.PrjPcb</t>
+  </si>
+  <si>
+    <t>7/19/2026</t>
+  </si>
+  <si>
+    <t>Samyar Sadat Akhavi</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>1746092-1</t>
+  </si>
+  <si>
+    <t>BAT54HT1G</t>
+  </si>
+  <si>
+    <t>BM02B-SRSS-TB(LF)(SN)</t>
+  </si>
+  <si>
+    <t>BQ41Z50RSNR</t>
+  </si>
+  <si>
+    <t>BQ296100DSGR</t>
+  </si>
+  <si>
+    <t>DMN1019USN-7</t>
+  </si>
+  <si>
+    <t>FDN358P</t>
+  </si>
+  <si>
+    <t>GEN-CC1UT10V25KX7R805</t>
+  </si>
+  <si>
+    <t>GEN-CC100NT10V25KX7R603</t>
+  </si>
+  <si>
+    <t>GEN-CC470NT10V16KX7R603</t>
+  </si>
+  <si>
+    <t>GEN-CILAMBLCLR805</t>
+  </si>
+  <si>
+    <t>GEN-CILGRNLCLR805</t>
+  </si>
+  <si>
+    <t>GEN-CILREDLCLR805</t>
+  </si>
+  <si>
+    <t>GEN-CRR1KT1P8603</t>
+  </si>
+  <si>
+    <t>GEN-CRR5K1T5P8603</t>
+  </si>
+  <si>
+    <t>GEN-CRR5R1T1P8603</t>
+  </si>
+  <si>
+    <t>GEN-CRR10KT5P8603</t>
+  </si>
+  <si>
+    <t>GEN-CRR10MT5P8603</t>
+  </si>
+  <si>
+    <t>GEN-CRR47T1P8603</t>
+  </si>
+  <si>
+    <t>GEN-CRR50T1P11206</t>
+  </si>
+  <si>
+    <t>GEN-CRR51KT5P8603</t>
+  </si>
+  <si>
+    <t>GEN-CRR100T1P8603</t>
+  </si>
+  <si>
+    <t>GEN-CRR300T5P8603</t>
+  </si>
+  <si>
+    <t>IQEH54NE2LM7UCG</t>
+  </si>
+  <si>
+    <t>IRLML6344TRPBF</t>
+  </si>
+  <si>
+    <t>ITV4030L1215</t>
+  </si>
+  <si>
+    <t>NTCGS163JX103DT8</t>
+  </si>
+  <si>
+    <t>PTS815SJK250SMTRLFS</t>
+  </si>
+  <si>
+    <t>S4B-XH-SM4-TB(LF)(SN)</t>
+  </si>
+  <si>
+    <t>SMCJ13A</t>
+  </si>
+  <si>
+    <t>TLR3A20DR001FTDG</t>
+  </si>
+  <si>
+    <t>TPD1E10B06DPYR</t>
+  </si>
+  <si>
+    <t>TPS70933DBVR</t>
+  </si>
+  <si>
+    <t>XT60PW-M</t>
+  </si>
+  <si>
+    <t>DIODE SCHOTTKY 30V 200MA SOD323</t>
+  </si>
+  <si>
+    <t>CONN HEADER SMD 2POS 1MM</t>
+  </si>
+  <si>
+    <t>2 TO 4 SERIES LI-ION HIGHLY INTE</t>
+  </si>
+  <si>
+    <t>IC BATT PROT LI-ION 2-4CEL 8WSON</t>
+  </si>
+  <si>
+    <t>MOSFET N-CH 12V 9.3A SC59</t>
+  </si>
+  <si>
+    <t>MOSFET P-CH 30V 1.5A SSOT3</t>
+  </si>
+  <si>
+    <t>GENERIC 0805 MLC CAPACITOR</t>
+  </si>
+  <si>
+    <t>GENERIC 0603 MLC CAPACITOR</t>
+  </si>
+  <si>
+    <t>GENERIC 0805 INDICATOR LED</t>
+  </si>
+  <si>
+    <t>GENERIC 0603 CHIP RESISTOR</t>
+  </si>
+  <si>
+    <t>GENERIC 1206 CHIP RESISTOR</t>
+  </si>
+  <si>
+    <t>IGFET, N-CHANNEL, ENHANCEMENT, BODY DIODE</t>
+  </si>
+  <si>
+    <t>MOSFET N-CH 30V 5A MICRO3/SOT23</t>
+  </si>
+  <si>
+    <t>FUSE BATTERY PROTECTOR 12V 15A</t>
+  </si>
+  <si>
+    <t>NTC,10K,0.5%,0603,150C,AEC-Q200,</t>
+  </si>
+  <si>
+    <t>SWITCH TACTILE SPST-NO 0.05A 12V</t>
+  </si>
+  <si>
+    <t>CONN HEADER SMD R/A 4POS 2.5MM</t>
+  </si>
+  <si>
+    <t>TVS DIODE 13VWM 21.5VC DO214AB</t>
+  </si>
+  <si>
+    <t>RES 0.001 OHM 1% 2W 2512</t>
+  </si>
+  <si>
+    <t>TVS DIODE 5.5VWM 14VC 2X1SON</t>
+  </si>
+  <si>
+    <t>IC REG LINEAR 3.3V 150MA SOT23-5</t>
+  </si>
+  <si>
+    <t>MALE XT60 PCB-MOUNT SOLDERABLE CONNECTOR</t>
+  </si>
+  <si>
     <t>100nF</t>
   </si>
   <si>
-    <t>25V</t>
+    <t>470nF</t>
+  </si>
+  <si>
+    <t>1k</t>
+  </si>
+  <si>
+    <t>5.1k</t>
+  </si>
+  <si>
+    <t>5.1R</t>
+  </si>
+  <si>
+    <t>10k</t>
+  </si>
+  <si>
+    <t>10M</t>
+  </si>
+  <si>
+    <t>47R</t>
+  </si>
+  <si>
+    <t>50R</t>
+  </si>
+  <si>
+    <t>51k</t>
+  </si>
+  <si>
+    <t>100R</t>
+  </si>
+  <si>
+    <t>300R</t>
+  </si>
+  <si>
+    <t>1 mOhms</t>
+  </si>
+  <si>
+    <t>16V</t>
+  </si>
+  <si>
+    <t>36VDC</t>
+  </si>
+  <si>
+    <t>±1%</t>
+  </si>
+  <si>
+    <t>±5%</t>
   </si>
   <si>
     <t>Green</t>
   </si>
   <si>
-    <t>GENERIC 0603 MLC CAPACITOR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Variant: </t>
-  </si>
-  <si>
-    <t>Part Number</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Tolerance</t>
-  </si>
-  <si>
-    <t>Voltage</t>
-  </si>
-  <si>
-    <t>Color</t>
-  </si>
-  <si>
-    <t>Quantity</t>
-  </si>
-  <si>
-    <t>Manufacturer</t>
-  </si>
-  <si>
-    <t>Supplier</t>
-  </si>
-  <si>
-    <t>Supplier Part Number</t>
-  </si>
-  <si>
-    <t>±10%</t>
+    <t>Red</t>
+  </si>
+  <si>
+    <t>ON Semiconductor</t>
+  </si>
+  <si>
+    <t>JST Sales America Inc.</t>
   </si>
   <si>
     <t>Texas Instruments</t>
   </si>
   <si>
-    <t>The ROS Robot Project</t>
-  </si>
-  <si>
-    <t>Pack_BMS_Module.PrjPcb</t>
-  </si>
-  <si>
-    <t>6/18/2026</t>
-  </si>
-  <si>
-    <t>Samyar Sadat Akhavi</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>GEN-CC100NT10V25KX7R603</t>
-  </si>
-  <si>
-    <t>GEN-CC1UT10V25KX7R603</t>
-  </si>
-  <si>
-    <t>GEN-CC470NT10V16KX7R603</t>
-  </si>
-  <si>
-    <t>TPD1E10B06DPYR</t>
-  </si>
-  <si>
-    <t>SMDJ13A</t>
-  </si>
-  <si>
-    <t>BAT54HT1G</t>
-  </si>
-  <si>
-    <t>GEN-CILGRNLCLR805</t>
-  </si>
-  <si>
-    <t>GEN-CILAMBLCLR805</t>
-  </si>
-  <si>
-    <t>GEN-CILREDLCLR805</t>
-  </si>
-  <si>
-    <t>ITV4030L1215</t>
-  </si>
-  <si>
-    <t>FDN358P</t>
-  </si>
-  <si>
-    <t>IRLML6344TRPBF</t>
-  </si>
-  <si>
-    <t>DMN1019USN-7</t>
-  </si>
-  <si>
-    <t>TPS70933DBVR</t>
-  </si>
-  <si>
-    <t>BM02B-SRSS-TB(LF)(SN)</t>
-  </si>
-  <si>
-    <t>S4B-XH-SM4-TB(LF)(SN)</t>
-  </si>
-  <si>
-    <t>XT60PW-M</t>
-  </si>
-  <si>
-    <t>1746092-1</t>
-  </si>
-  <si>
-    <t>IQEH54NE2LM7UCG</t>
-  </si>
-  <si>
-    <t>GEN-CRR100T1P8603</t>
-  </si>
-  <si>
-    <t>GEN-CRR47T1P8603</t>
-  </si>
-  <si>
-    <t>GEN-CRR300T5P8603</t>
-  </si>
-  <si>
-    <t>GEN-CRR10MT5P8603</t>
-  </si>
-  <si>
-    <t>GEN-CRR10KT5P8603</t>
-  </si>
-  <si>
-    <t>GEN-CRR5K1T5P8603</t>
-  </si>
-  <si>
-    <t>GEN-CRR51KT5P8603</t>
-  </si>
-  <si>
-    <t>GEN-CRR1KT1P8603</t>
-  </si>
-  <si>
-    <t>GEN-CRR50T1P11206</t>
-  </si>
-  <si>
-    <t>TLR3A20DR001FTDG</t>
-  </si>
-  <si>
-    <t>GEN-CRR5R1T1P8603</t>
-  </si>
-  <si>
-    <t>PTS815SJK250SMTRLFS</t>
-  </si>
-  <si>
-    <t>BQ41Z50RSNR</t>
-  </si>
-  <si>
-    <t>BQ296100DSGR</t>
-  </si>
-  <si>
-    <t>TVS DIODE 5.5VWM 14VC 2X1SON</t>
-  </si>
-  <si>
-    <t>TVS DIODE 13VWM 21.5VC DO214AB</t>
-  </si>
-  <si>
-    <t>DIODE SCHOTTKY 30V 200MA SOD323</t>
-  </si>
-  <si>
-    <t>GENERIC 0805 INDICATOR LED</t>
-  </si>
-  <si>
-    <t>FUSE BATTERY PROTECTOR 12V 15A</t>
-  </si>
-  <si>
-    <t>MOSFET P-CH 30V 1.5A SSOT3</t>
-  </si>
-  <si>
-    <t>MOSFET N-CH 30V 5A MICRO3/SOT23</t>
-  </si>
-  <si>
-    <t>MOSFET N-CH 12V 9.3A SC59</t>
-  </si>
-  <si>
-    <t>IC REG LINEAR 3.3V 150MA SOT23-5</t>
-  </si>
-  <si>
-    <t>CONN HEADER SMD 2POS 1MM</t>
-  </si>
-  <si>
-    <t>CONN HEADER SMD R/A 4POS 2.5MM</t>
-  </si>
-  <si>
-    <t>MALE XT60 PCB-MOUNT SOLDERABLE CONNECTOR</t>
-  </si>
-  <si>
-    <t>CONN PLUG 10POS 2.50MM R/A SLDR</t>
-  </si>
-  <si>
-    <t>IGFET, N-CHANNEL, ENHANCEMENT, BODY DIODE</t>
-  </si>
-  <si>
-    <t>GENERIC 0603 CHIP RESISTOR</t>
-  </si>
-  <si>
-    <t>GENERIC 1206 CHIP RESISTOR</t>
-  </si>
-  <si>
-    <t>RES 0.001 OHM 1% 2W 2512</t>
-  </si>
-  <si>
-    <t>SWITCH TACTILE SPST-NO 0.05A 12V</t>
-  </si>
-  <si>
-    <t>2 TO 4 SERIES LI-ION HIGHLY INTE</t>
-  </si>
-  <si>
-    <t>IC BATT PROT LI-ION 2-4CEL 8WSON</t>
-  </si>
-  <si>
-    <t>1µF</t>
-  </si>
-  <si>
-    <t>470nF</t>
-  </si>
-  <si>
-    <t>100R</t>
-  </si>
-  <si>
-    <t>47R</t>
-  </si>
-  <si>
-    <t>300R</t>
-  </si>
-  <si>
-    <t>10M</t>
-  </si>
-  <si>
-    <t>10k</t>
-  </si>
-  <si>
-    <t>5.1k</t>
-  </si>
-  <si>
-    <t>51k</t>
-  </si>
-  <si>
-    <t>1k</t>
-  </si>
-  <si>
-    <t>50R</t>
-  </si>
-  <si>
-    <t>1 mOhms</t>
-  </si>
-  <si>
-    <t>5.1R</t>
-  </si>
-  <si>
-    <t>16V</t>
-  </si>
-  <si>
-    <t>36VDC</t>
-  </si>
-  <si>
-    <t>±1%</t>
-  </si>
-  <si>
-    <t>±5%</t>
-  </si>
-  <si>
-    <t>Amber</t>
-  </si>
-  <si>
-    <t>Red</t>
+    <t>Diodes Incorporated</t>
+  </si>
+  <si>
+    <t>Infineon Technologies</t>
   </si>
   <si>
     <t>Littelfuse Inc.</t>
   </si>
   <si>
-    <t>ON Semiconductor</t>
-  </si>
-  <si>
-    <t>Infineon Technologies</t>
-  </si>
-  <si>
-    <t>Diodes Incorporated</t>
-  </si>
-  <si>
-    <t>JST Sales America Inc.</t>
+    <t>TDK Corporation</t>
+  </si>
+  <si>
+    <t>C&amp;K</t>
+  </si>
+  <si>
+    <t>TE Connectivity Passive Product</t>
   </si>
   <si>
     <t>AMASS</t>
   </si>
   <si>
-    <t>TE Connectivity AMP Connectors</t>
-  </si>
-  <si>
-    <t>TE Connectivity Passive Product</t>
-  </si>
-  <si>
-    <t>C&amp;K</t>
-  </si>
-  <si>
     <t>DigiKey</t>
   </si>
   <si>
     <t>TME</t>
   </si>
   <si>
+    <t>A107791-ND</t>
+  </si>
+  <si>
+    <t>BAT54HT1GOSCT-ND</t>
+  </si>
+  <si>
+    <t>455-1788-1-ND</t>
+  </si>
+  <si>
+    <t>296-BQ41Z50RSNRCT-ND</t>
+  </si>
+  <si>
+    <t>296-50964-1-ND</t>
+  </si>
+  <si>
+    <t>DMN1019USN-7DICT-ND</t>
+  </si>
+  <si>
+    <t>FDN358PCT-ND</t>
+  </si>
+  <si>
+    <t>448-IQEH54NE2LM7UCGATMA1CT-ND</t>
+  </si>
+  <si>
+    <t>IRLML6344TRPBFCT-ND</t>
+  </si>
+  <si>
+    <t>18-ITV4030L1215NRCT-ND</t>
+  </si>
+  <si>
+    <t>445-NTCGS163JX103DT8CT-ND</t>
+  </si>
+  <si>
+    <t>CKN12216-1-ND</t>
+  </si>
+  <si>
+    <t>455-2262-1-ND</t>
+  </si>
+  <si>
+    <t>SMCJ13ALFCT-ND</t>
+  </si>
+  <si>
+    <t>A129565CT-ND</t>
+  </si>
+  <si>
     <t>296-30406-1-ND</t>
   </si>
   <si>
-    <t>SMDJ13ACT-ND</t>
-  </si>
-  <si>
-    <t>BAT54HT1GOSCT-ND</t>
-  </si>
-  <si>
-    <t>18-ITV4030L1215NRCT-ND</t>
-  </si>
-  <si>
-    <t>FDN358PCT-ND</t>
-  </si>
-  <si>
-    <t>IRLML6344TRPBFCT-ND</t>
-  </si>
-  <si>
-    <t>DMN1019USN-7DICT-ND</t>
-  </si>
-  <si>
     <t>296-35483-1-ND</t>
-  </si>
-  <si>
-    <t>455-1788-1-ND</t>
-  </si>
-  <si>
-    <t>455-2262-1-ND</t>
-  </si>
-  <si>
-    <t>A107791-ND</t>
-  </si>
-  <si>
-    <t>448-IQEH54NE2LM7UCGATMA1CT-ND</t>
-  </si>
-  <si>
-    <t>A129565CT-ND</t>
-  </si>
-  <si>
-    <t>CKN12216-1-ND</t>
-  </si>
-  <si>
-    <t>296-BQ41Z50RSNRCT-ND</t>
-  </si>
-  <si>
-    <t>296-50964-1-ND</t>
   </si>
 </sst>
 </file>
@@ -1365,7 +1380,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:K50"/>
   <sheetFormatPr defaultRowHeight="15" baseColWidth="0"/>
   <cols>
     <col min="1" max="1" width="4.99609375" customWidth="1"/>
@@ -1558,21 +1573,21 @@
       <c r="C13" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="D13" s="26" t="s">
-        <v>7</v>
-      </c>
-      <c r="E13" s="26" t="s">
-        <v>8</v>
-      </c>
-      <c r="F13" s="26" t="s">
-        <v>22</v>
-      </c>
+      <c r="D13" s="26"/>
+      <c r="E13" s="26"/>
+      <c r="F13" s="26"/>
       <c r="G13" s="26"/>
-      <c r="H13" s="26"/>
-      <c r="I13" s="26"/>
-      <c r="J13" s="26"/>
+      <c r="H13" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="I13" s="26" t="s">
+        <v>114</v>
+      </c>
+      <c r="J13" s="26" t="s">
+        <v>116</v>
+      </c>
       <c r="K13" s="27">
-        <v>21</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="2:11">
@@ -1580,23 +1595,23 @@
         <v>30</v>
       </c>
       <c r="C14" s="29" t="s">
-        <v>10</v>
-      </c>
-      <c r="D14" s="26" t="s">
-        <v>82</v>
-      </c>
-      <c r="E14" s="26" t="s">
-        <v>8</v>
-      </c>
-      <c r="F14" s="26" t="s">
-        <v>22</v>
-      </c>
+        <v>63</v>
+      </c>
+      <c r="D14" s="26"/>
+      <c r="E14" s="26"/>
+      <c r="F14" s="26"/>
       <c r="G14" s="26"/>
-      <c r="H14" s="26"/>
-      <c r="I14" s="26"/>
-      <c r="J14" s="26"/>
+      <c r="H14" s="26" t="s">
+        <v>104</v>
+      </c>
+      <c r="I14" s="26" t="s">
+        <v>114</v>
+      </c>
+      <c r="J14" s="26" t="s">
+        <v>117</v>
+      </c>
       <c r="K14" s="27">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="2:11" customHeight="1" thickBot="1">
@@ -1604,23 +1619,23 @@
         <v>31</v>
       </c>
       <c r="C15" s="29" t="s">
-        <v>10</v>
-      </c>
-      <c r="D15" s="26" t="s">
-        <v>83</v>
-      </c>
-      <c r="E15" s="26" t="s">
-        <v>95</v>
-      </c>
-      <c r="F15" s="26" t="s">
-        <v>22</v>
-      </c>
+        <v>64</v>
+      </c>
+      <c r="D15" s="26"/>
+      <c r="E15" s="26"/>
+      <c r="F15" s="26"/>
       <c r="G15" s="26"/>
-      <c r="H15" s="26"/>
-      <c r="I15" s="26"/>
-      <c r="J15" s="26"/>
+      <c r="H15" s="26" t="s">
+        <v>105</v>
+      </c>
+      <c r="I15" s="26" t="s">
+        <v>114</v>
+      </c>
+      <c r="J15" s="26" t="s">
+        <v>118</v>
+      </c>
       <c r="K15" s="27">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16" spans="2:11" customHeight="1" thickBot="1">
@@ -1628,23 +1643,23 @@
         <v>32</v>
       </c>
       <c r="C16" s="29" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D16" s="26"/>
       <c r="E16" s="26"/>
       <c r="F16" s="26"/>
       <c r="G16" s="26"/>
       <c r="H16" s="26" t="s">
-        <v>23</v>
+        <v>106</v>
       </c>
       <c r="I16" s="26" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="J16" s="26" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="K16" s="27">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="2:11" customHeight="1" thickBot="1">
@@ -1652,20 +1667,20 @@
         <v>33</v>
       </c>
       <c r="C17" s="29" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="D17" s="26"/>
       <c r="E17" s="26"/>
       <c r="F17" s="26"/>
       <c r="G17" s="26"/>
       <c r="H17" s="26" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="I17" s="26" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="J17" s="26" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="K17" s="27">
         <v>1</v>
@@ -1676,23 +1691,23 @@
         <v>34</v>
       </c>
       <c r="C18" s="29" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D18" s="26"/>
       <c r="E18" s="26"/>
       <c r="F18" s="26"/>
       <c r="G18" s="26"/>
       <c r="H18" s="26" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="I18" s="26" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="J18" s="26" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="K18" s="27">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="2:11" customHeight="1" thickBot="1">
@@ -1700,17 +1715,21 @@
         <v>35</v>
       </c>
       <c r="C19" s="29" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="D19" s="26"/>
       <c r="E19" s="26"/>
       <c r="F19" s="26"/>
-      <c r="G19" s="26" t="s">
-        <v>9</v>
-      </c>
-      <c r="H19" s="26"/>
-      <c r="I19" s="26"/>
-      <c r="J19" s="26"/>
+      <c r="G19" s="26"/>
+      <c r="H19" s="26" t="s">
+        <v>104</v>
+      </c>
+      <c r="I19" s="26" t="s">
+        <v>114</v>
+      </c>
+      <c r="J19" s="26" t="s">
+        <v>122</v>
+      </c>
       <c r="K19" s="27">
         <v>1</v>
       </c>
@@ -1720,19 +1739,23 @@
         <v>36</v>
       </c>
       <c r="C20" s="29" t="s">
-        <v>65</v>
-      </c>
-      <c r="D20" s="26"/>
-      <c r="E20" s="26"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="26" t="s">
-        <v>99</v>
-      </c>
+        <v>69</v>
+      </c>
+      <c r="D20" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="E20" s="26" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" s="26" t="s">
+        <v>22</v>
+      </c>
+      <c r="G20" s="26"/>
       <c r="H20" s="26"/>
       <c r="I20" s="26"/>
       <c r="J20" s="26"/>
       <c r="K20" s="27">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21" spans="2:11" customHeight="1" thickBot="1">
@@ -1740,19 +1763,23 @@
         <v>37</v>
       </c>
       <c r="C21" s="29" t="s">
-        <v>65</v>
-      </c>
-      <c r="D21" s="26"/>
-      <c r="E21" s="26"/>
-      <c r="F21" s="26"/>
-      <c r="G21" s="26" t="s">
-        <v>100</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="D21" s="26" t="s">
+        <v>85</v>
+      </c>
+      <c r="E21" s="26" t="s">
+        <v>8</v>
+      </c>
+      <c r="F21" s="26" t="s">
+        <v>22</v>
+      </c>
+      <c r="G21" s="26"/>
       <c r="H21" s="26"/>
       <c r="I21" s="26"/>
       <c r="J21" s="26"/>
       <c r="K21" s="27">
-        <v>1</v>
+        <v>21</v>
       </c>
     </row>
     <row r="22" spans="2:11" customHeight="1" thickBot="1">
@@ -1760,23 +1787,21 @@
         <v>38</v>
       </c>
       <c r="C22" s="29" t="s">
-        <v>66</v>
-      </c>
-      <c r="D22" s="26"/>
+        <v>70</v>
+      </c>
+      <c r="D22" s="26" t="s">
+        <v>86</v>
+      </c>
       <c r="E22" s="26" t="s">
-        <v>96</v>
-      </c>
-      <c r="F22" s="26"/>
+        <v>98</v>
+      </c>
+      <c r="F22" s="26" t="s">
+        <v>22</v>
+      </c>
       <c r="G22" s="26"/>
-      <c r="H22" s="26" t="s">
-        <v>101</v>
-      </c>
-      <c r="I22" s="26" t="s">
-        <v>110</v>
-      </c>
-      <c r="J22" s="26" t="s">
-        <v>115</v>
-      </c>
+      <c r="H22" s="26"/>
+      <c r="I22" s="26"/>
+      <c r="J22" s="26"/>
       <c r="K22" s="27">
         <v>1</v>
       </c>
@@ -1786,21 +1811,17 @@
         <v>39</v>
       </c>
       <c r="C23" s="29" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="D23" s="26"/>
       <c r="E23" s="26"/>
       <c r="F23" s="26"/>
-      <c r="G23" s="26"/>
-      <c r="H23" s="26" t="s">
-        <v>102</v>
-      </c>
-      <c r="I23" s="26" t="s">
-        <v>110</v>
-      </c>
-      <c r="J23" s="26" t="s">
-        <v>116</v>
-      </c>
+      <c r="G23" s="26" t="s">
+        <v>9</v>
+      </c>
+      <c r="H23" s="26"/>
+      <c r="I23" s="26"/>
+      <c r="J23" s="26"/>
       <c r="K23" s="27">
         <v>1</v>
       </c>
@@ -1810,23 +1831,19 @@
         <v>40</v>
       </c>
       <c r="C24" s="29" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D24" s="26"/>
       <c r="E24" s="26"/>
       <c r="F24" s="26"/>
-      <c r="G24" s="26"/>
-      <c r="H24" s="26" t="s">
-        <v>103</v>
-      </c>
-      <c r="I24" s="26" t="s">
-        <v>110</v>
-      </c>
-      <c r="J24" s="26" t="s">
-        <v>117</v>
-      </c>
+      <c r="G24" s="26" t="s">
+        <v>102</v>
+      </c>
+      <c r="H24" s="26"/>
+      <c r="I24" s="26"/>
+      <c r="J24" s="26"/>
       <c r="K24" s="27">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="2:11" customHeight="1" thickBot="1">
@@ -1834,23 +1851,19 @@
         <v>41</v>
       </c>
       <c r="C25" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D25" s="26"/>
       <c r="E25" s="26"/>
       <c r="F25" s="26"/>
-      <c r="G25" s="26"/>
-      <c r="H25" s="26" t="s">
-        <v>104</v>
-      </c>
-      <c r="I25" s="26" t="s">
-        <v>110</v>
-      </c>
-      <c r="J25" s="26" t="s">
-        <v>118</v>
-      </c>
+      <c r="G25" s="26" t="s">
+        <v>103</v>
+      </c>
+      <c r="H25" s="26"/>
+      <c r="I25" s="26"/>
+      <c r="J25" s="26"/>
       <c r="K25" s="27">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="2:11" customHeight="1" thickBot="1">
@@ -1858,23 +1871,21 @@
         <v>42</v>
       </c>
       <c r="C26" s="29" t="s">
-        <v>70</v>
-      </c>
-      <c r="D26" s="26"/>
+        <v>72</v>
+      </c>
+      <c r="D26" s="26" t="s">
+        <v>87</v>
+      </c>
       <c r="E26" s="26"/>
-      <c r="F26" s="26"/>
+      <c r="F26" s="26" t="s">
+        <v>100</v>
+      </c>
       <c r="G26" s="26"/>
-      <c r="H26" s="26" t="s">
-        <v>23</v>
-      </c>
-      <c r="I26" s="26" t="s">
-        <v>110</v>
-      </c>
-      <c r="J26" s="26" t="s">
-        <v>119</v>
-      </c>
+      <c r="H26" s="26"/>
+      <c r="I26" s="26"/>
+      <c r="J26" s="26"/>
       <c r="K26" s="27">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="27" spans="2:11" customHeight="1" thickBot="1">
@@ -1882,23 +1893,21 @@
         <v>43</v>
       </c>
       <c r="C27" s="29" t="s">
-        <v>71</v>
-      </c>
-      <c r="D27" s="26"/>
+        <v>72</v>
+      </c>
+      <c r="D27" s="26" t="s">
+        <v>88</v>
+      </c>
       <c r="E27" s="26"/>
-      <c r="F27" s="26"/>
+      <c r="F27" s="26" t="s">
+        <v>101</v>
+      </c>
       <c r="G27" s="26"/>
-      <c r="H27" s="26" t="s">
-        <v>105</v>
-      </c>
-      <c r="I27" s="26" t="s">
-        <v>110</v>
-      </c>
-      <c r="J27" s="26" t="s">
-        <v>120</v>
-      </c>
+      <c r="H27" s="26"/>
+      <c r="I27" s="26"/>
+      <c r="J27" s="26"/>
       <c r="K27" s="27">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28" spans="2:11" customHeight="1" thickBot="1">
@@ -1908,19 +1917,17 @@
       <c r="C28" s="29" t="s">
         <v>72</v>
       </c>
-      <c r="D28" s="26"/>
+      <c r="D28" s="26" t="s">
+        <v>89</v>
+      </c>
       <c r="E28" s="26"/>
-      <c r="F28" s="26"/>
+      <c r="F28" s="26" t="s">
+        <v>100</v>
+      </c>
       <c r="G28" s="26"/>
-      <c r="H28" s="26" t="s">
-        <v>105</v>
-      </c>
-      <c r="I28" s="26" t="s">
-        <v>110</v>
-      </c>
-      <c r="J28" s="26" t="s">
-        <v>121</v>
-      </c>
+      <c r="H28" s="26"/>
+      <c r="I28" s="26"/>
+      <c r="J28" s="26"/>
       <c r="K28" s="27">
         <v>1</v>
       </c>
@@ -1930,23 +1937,21 @@
         <v>45</v>
       </c>
       <c r="C29" s="29" t="s">
-        <v>73</v>
-      </c>
-      <c r="D29" s="26"/>
+        <v>72</v>
+      </c>
+      <c r="D29" s="26" t="s">
+        <v>90</v>
+      </c>
       <c r="E29" s="26"/>
-      <c r="F29" s="26"/>
+      <c r="F29" s="26" t="s">
+        <v>101</v>
+      </c>
       <c r="G29" s="26"/>
-      <c r="H29" s="26" t="s">
-        <v>106</v>
-      </c>
-      <c r="I29" s="26" t="s">
-        <v>111</v>
-      </c>
-      <c r="J29" s="26" t="s">
-        <v>45</v>
-      </c>
+      <c r="H29" s="26"/>
+      <c r="I29" s="26"/>
+      <c r="J29" s="26"/>
       <c r="K29" s="27">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30" spans="2:11" customHeight="1" thickBot="1">
@@ -1954,23 +1959,21 @@
         <v>46</v>
       </c>
       <c r="C30" s="29" t="s">
-        <v>74</v>
-      </c>
-      <c r="D30" s="26"/>
+        <v>72</v>
+      </c>
+      <c r="D30" s="26" t="s">
+        <v>91</v>
+      </c>
       <c r="E30" s="26"/>
-      <c r="F30" s="26"/>
+      <c r="F30" s="26" t="s">
+        <v>101</v>
+      </c>
       <c r="G30" s="26"/>
-      <c r="H30" s="26" t="s">
-        <v>107</v>
-      </c>
-      <c r="I30" s="26" t="s">
-        <v>110</v>
-      </c>
-      <c r="J30" s="26" t="s">
-        <v>122</v>
-      </c>
+      <c r="H30" s="26"/>
+      <c r="I30" s="26"/>
+      <c r="J30" s="26"/>
       <c r="K30" s="27">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31" spans="2:11" customHeight="1" thickBot="1">
@@ -1978,23 +1981,21 @@
         <v>47</v>
       </c>
       <c r="C31" s="29" t="s">
-        <v>75</v>
-      </c>
-      <c r="D31" s="26"/>
+        <v>72</v>
+      </c>
+      <c r="D31" s="26" t="s">
+        <v>92</v>
+      </c>
       <c r="E31" s="26"/>
-      <c r="F31" s="26"/>
+      <c r="F31" s="26" t="s">
+        <v>100</v>
+      </c>
       <c r="G31" s="26"/>
-      <c r="H31" s="26" t="s">
-        <v>103</v>
-      </c>
-      <c r="I31" s="26" t="s">
-        <v>110</v>
-      </c>
-      <c r="J31" s="26" t="s">
-        <v>123</v>
-      </c>
+      <c r="H31" s="26"/>
+      <c r="I31" s="26"/>
+      <c r="J31" s="26"/>
       <c r="K31" s="27">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32" spans="2:11" customHeight="1" thickBot="1">
@@ -2002,21 +2003,21 @@
         <v>48</v>
       </c>
       <c r="C32" s="29" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D32" s="26" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="E32" s="26"/>
       <c r="F32" s="26" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="G32" s="26"/>
       <c r="H32" s="26"/>
       <c r="I32" s="26"/>
       <c r="J32" s="26"/>
       <c r="K32" s="27">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33" spans="2:11" customHeight="1" thickBot="1">
@@ -2024,21 +2025,21 @@
         <v>49</v>
       </c>
       <c r="C33" s="29" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="D33" s="26" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="E33" s="26"/>
       <c r="F33" s="26" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G33" s="26"/>
       <c r="H33" s="26"/>
       <c r="I33" s="26"/>
       <c r="J33" s="26"/>
       <c r="K33" s="27">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" spans="2:11" customHeight="1" thickBot="1">
@@ -2046,21 +2047,21 @@
         <v>50</v>
       </c>
       <c r="C34" s="29" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="D34" s="26" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="E34" s="26"/>
       <c r="F34" s="26" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G34" s="26"/>
       <c r="H34" s="26"/>
       <c r="I34" s="26"/>
       <c r="J34" s="26"/>
       <c r="K34" s="27">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="35" spans="2:11" customHeight="1" thickBot="1">
@@ -2068,21 +2069,21 @@
         <v>51</v>
       </c>
       <c r="C35" s="29" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="D35" s="26" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="E35" s="26"/>
       <c r="F35" s="26" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="G35" s="26"/>
       <c r="H35" s="26"/>
       <c r="I35" s="26"/>
       <c r="J35" s="26"/>
       <c r="K35" s="27">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="2:11" customHeight="1" thickBot="1">
@@ -2090,19 +2091,21 @@
         <v>52</v>
       </c>
       <c r="C36" s="29" t="s">
-        <v>76</v>
-      </c>
-      <c r="D36" s="26" t="s">
-        <v>88</v>
-      </c>
+        <v>74</v>
+      </c>
+      <c r="D36" s="26"/>
       <c r="E36" s="26"/>
-      <c r="F36" s="26" t="s">
-        <v>98</v>
-      </c>
+      <c r="F36" s="26"/>
       <c r="G36" s="26"/>
-      <c r="H36" s="26"/>
-      <c r="I36" s="26"/>
-      <c r="J36" s="26"/>
+      <c r="H36" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="I36" s="26" t="s">
+        <v>114</v>
+      </c>
+      <c r="J36" s="26" t="s">
+        <v>123</v>
+      </c>
       <c r="K36" s="27">
         <v>2</v>
       </c>
@@ -2112,21 +2115,23 @@
         <v>53</v>
       </c>
       <c r="C37" s="29" t="s">
-        <v>76</v>
-      </c>
-      <c r="D37" s="26" t="s">
-        <v>89</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="D37" s="26"/>
       <c r="E37" s="26"/>
-      <c r="F37" s="26" t="s">
-        <v>98</v>
-      </c>
+      <c r="F37" s="26"/>
       <c r="G37" s="26"/>
-      <c r="H37" s="26"/>
-      <c r="I37" s="26"/>
-      <c r="J37" s="26"/>
+      <c r="H37" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="I37" s="26" t="s">
+        <v>114</v>
+      </c>
+      <c r="J37" s="26" t="s">
+        <v>124</v>
+      </c>
       <c r="K37" s="27">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38" spans="2:11" customHeight="1" thickBot="1">
@@ -2136,17 +2141,21 @@
       <c r="C38" s="29" t="s">
         <v>76</v>
       </c>
-      <c r="D38" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="E38" s="26"/>
-      <c r="F38" s="26" t="s">
-        <v>98</v>
-      </c>
+      <c r="D38" s="26"/>
+      <c r="E38" s="26" t="s">
+        <v>99</v>
+      </c>
+      <c r="F38" s="26"/>
       <c r="G38" s="26"/>
-      <c r="H38" s="26"/>
-      <c r="I38" s="26"/>
-      <c r="J38" s="26"/>
+      <c r="H38" s="26" t="s">
+        <v>109</v>
+      </c>
+      <c r="I38" s="26" t="s">
+        <v>114</v>
+      </c>
+      <c r="J38" s="26" t="s">
+        <v>125</v>
+      </c>
       <c r="K38" s="27">
         <v>1</v>
       </c>
@@ -2156,21 +2165,25 @@
         <v>55</v>
       </c>
       <c r="C39" s="29" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D39" s="26" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E39" s="26"/>
-      <c r="F39" s="26" t="s">
-        <v>97</v>
-      </c>
+      <c r="F39" s="26"/>
       <c r="G39" s="26"/>
-      <c r="H39" s="26"/>
-      <c r="I39" s="26"/>
-      <c r="J39" s="26"/>
+      <c r="H39" s="26" t="s">
+        <v>110</v>
+      </c>
+      <c r="I39" s="26" t="s">
+        <v>114</v>
+      </c>
+      <c r="J39" s="26" t="s">
+        <v>126</v>
+      </c>
       <c r="K39" s="27">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="2:11" customHeight="1" thickBot="1">
@@ -2178,21 +2191,23 @@
         <v>56</v>
       </c>
       <c r="C40" s="29" t="s">
-        <v>77</v>
-      </c>
-      <c r="D40" s="26" t="s">
-        <v>92</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="D40" s="26"/>
       <c r="E40" s="26"/>
-      <c r="F40" s="26" t="s">
-        <v>97</v>
-      </c>
+      <c r="F40" s="26"/>
       <c r="G40" s="26"/>
-      <c r="H40" s="26"/>
-      <c r="I40" s="26"/>
-      <c r="J40" s="26"/>
+      <c r="H40" s="26" t="s">
+        <v>111</v>
+      </c>
+      <c r="I40" s="26" t="s">
+        <v>114</v>
+      </c>
+      <c r="J40" s="26" t="s">
+        <v>127</v>
+      </c>
       <c r="K40" s="27">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41" spans="2:11" customHeight="1" thickBot="1">
@@ -2200,24 +2215,20 @@
         <v>57</v>
       </c>
       <c r="C41" s="29" t="s">
-        <v>78</v>
-      </c>
-      <c r="D41" s="26" t="s">
-        <v>93</v>
-      </c>
+        <v>79</v>
+      </c>
+      <c r="D41" s="26"/>
       <c r="E41" s="26"/>
-      <c r="F41" s="26" t="s">
-        <v>97</v>
-      </c>
+      <c r="F41" s="26"/>
       <c r="G41" s="26"/>
       <c r="H41" s="26" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="I41" s="26" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="J41" s="26" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="K41" s="27">
         <v>1</v>
@@ -2228,19 +2239,21 @@
         <v>58</v>
       </c>
       <c r="C42" s="29" t="s">
-        <v>76</v>
-      </c>
-      <c r="D42" s="26" t="s">
-        <v>94</v>
-      </c>
+        <v>80</v>
+      </c>
+      <c r="D42" s="26"/>
       <c r="E42" s="26"/>
-      <c r="F42" s="26" t="s">
-        <v>97</v>
-      </c>
+      <c r="F42" s="26"/>
       <c r="G42" s="26"/>
-      <c r="H42" s="26"/>
-      <c r="I42" s="26"/>
-      <c r="J42" s="26"/>
+      <c r="H42" s="26" t="s">
+        <v>109</v>
+      </c>
+      <c r="I42" s="26" t="s">
+        <v>114</v>
+      </c>
+      <c r="J42" s="26" t="s">
+        <v>129</v>
+      </c>
       <c r="K42" s="27">
         <v>1</v>
       </c>
@@ -2250,20 +2263,24 @@
         <v>59</v>
       </c>
       <c r="C43" s="29" t="s">
-        <v>79</v>
-      </c>
-      <c r="D43" s="26"/>
+        <v>81</v>
+      </c>
+      <c r="D43" s="26" t="s">
+        <v>97</v>
+      </c>
       <c r="E43" s="26"/>
-      <c r="F43" s="26"/>
+      <c r="F43" s="26" t="s">
+        <v>100</v>
+      </c>
       <c r="G43" s="26"/>
       <c r="H43" s="26" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="I43" s="26" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="J43" s="26" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="K43" s="27">
         <v>1</v>
@@ -2274,23 +2291,23 @@
         <v>60</v>
       </c>
       <c r="C44" s="29" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D44" s="26"/>
       <c r="E44" s="26"/>
       <c r="F44" s="26"/>
       <c r="G44" s="26"/>
       <c r="H44" s="26" t="s">
-        <v>23</v>
+        <v>106</v>
       </c>
       <c r="I44" s="26" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="J44" s="26" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="K44" s="27">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="45" spans="2:11" customHeight="1" thickBot="1">
@@ -2298,63 +2315,77 @@
         <v>61</v>
       </c>
       <c r="C45" s="29" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D45" s="26"/>
       <c r="E45" s="26"/>
       <c r="F45" s="26"/>
       <c r="G45" s="26"/>
       <c r="H45" s="26" t="s">
-        <v>23</v>
+        <v>106</v>
       </c>
       <c r="I45" s="26" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="J45" s="26" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="K45" s="27">
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="2:11">
-      <c r="B46" s="10"/>
-      <c r="C46" s="1"/>
-      <c r="D46" s="1"/>
-      <c r="E46" s="1"/>
-      <c r="F46" s="1"/>
-      <c r="G46" s="1"/>
-      <c r="H46" s="11"/>
-      <c r="I46" s="11"/>
-      <c r="J46" s="12"/>
-      <c r="K46" s="21" t="s">
+    <row r="46" spans="2:11" customHeight="1" thickBot="1">
+      <c r="B46" s="28" t="s">
+        <v>62</v>
+      </c>
+      <c r="C46" s="29" t="s">
+        <v>84</v>
+      </c>
+      <c r="D46" s="26"/>
+      <c r="E46" s="26"/>
+      <c r="F46" s="26"/>
+      <c r="G46" s="26"/>
+      <c r="H46" s="26" t="s">
+        <v>113</v>
+      </c>
+      <c r="I46" s="26" t="s">
+        <v>115</v>
+      </c>
+      <c r="J46" s="26" t="s">
+        <v>62</v>
+      </c>
+      <c r="K46" s="27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="2:11">
+      <c r="B47" s="10"/>
+      <c r="C47" s="1"/>
+      <c r="D47" s="1"/>
+      <c r="E47" s="1"/>
+      <c r="F47" s="1"/>
+      <c r="G47" s="1"/>
+      <c r="H47" s="11"/>
+      <c r="I47" s="11"/>
+      <c r="J47" s="12"/>
+      <c r="K47" s="21" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="47" spans="2:11" ht="15.75" thickBot="1">
-      <c r="B47" s="8"/>
-      <c r="C47" s="3"/>
-      <c r="D47" s="3"/>
-      <c r="E47" s="3"/>
-      <c r="F47" s="3"/>
-      <c r="G47" s="3"/>
-      <c r="H47" s="4"/>
-      <c r="I47" s="4"/>
-      <c r="J47" s="9"/>
-      <c r="K47" s="20">
-        <f>SUM(K13:K45)</f>
+    <row r="48" spans="2:11" ht="15.75" thickBot="1">
+      <c r="B48" s="8"/>
+      <c r="C48" s="3"/>
+      <c r="D48" s="3"/>
+      <c r="E48" s="3"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="4"/>
+      <c r="I48" s="4"/>
+      <c r="J48" s="9"/>
+      <c r="K48" s="20">
+        <f>SUM(K13:K46)</f>
         <v>87</v>
       </c>
-    </row>
-    <row r="48" spans="2:9">
-      <c r="B48"/>
-      <c r="C48"/>
-      <c r="D48"/>
-      <c r="E48"/>
-      <c r="F48"/>
-      <c r="G48"/>
-      <c r="H48"/>
-      <c r="I48"/>
     </row>
     <row r="49" spans="2:9">
       <c r="B49"/>
@@ -2366,6 +2397,16 @@
       <c r="H49"/>
       <c r="I49"/>
     </row>
+    <row r="50" spans="2:9">
+      <c r="B50"/>
+      <c r="C50"/>
+      <c r="D50"/>
+      <c r="E50"/>
+      <c r="F50"/>
+      <c r="G50"/>
+      <c r="H50"/>
+      <c r="I50"/>
+    </row>
   </sheetData>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="85" orientation="landscape" r:id="rId1"/>

</xml_diff>